<commit_message>
Dissertação: pareceres da banca e análise comentário a comentário
Guarda o trabalho revisado (.docx) e os dois pareceres em PDF (Fernando e
Marcos Bernardes) em dissertacao_PSN/banca/, com a análise de cada um dos
109 comentários: o que pede, opinião e proposta de texto para aprovação.
Inclui a comparação de graus polinomiais 1 a 5 com a base 2001-2025
(grau 2 ótimo nos três biomas), suas figuras e a atualização do
RESULTADOS.md.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018VBB2nFu5nBvcdBQC7zcsW
</commit_message>
<xml_diff>
--- a/dissertacao_PSN/Dados_base_nova_2001_2025.xlsx
+++ b/dissertacao_PSN/Dados_base_nova_2001_2025.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>